<commit_message>
Add PV load curve
</commit_message>
<xml_diff>
--- a/grodent-magnenat-mini-projet-trey/input-data/load_curve/power_profile_cabinet_summer_week.xlsx
+++ b/grodent-magnenat-mini-projet-trey/input-data/load_curve/power_profile_cabinet_summer_week.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\max\github\rhtlab\grodent-magnenat-mini-projet-trey\input-data\load_curve\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC465387-EF23-46CE-8481-1C190EF93BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{156464E3-1D3B-4709-90A0-ECAD2CC9D71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="26537" windowHeight="15943" xr2:uid="{5FC146A3-AC37-46DC-AD92-E888F69598AC}"/>
+    <workbookView xWindow="720" yWindow="720" windowWidth="20983" windowHeight="14794" activeTab="1" xr2:uid="{5FC146A3-AC37-46DC-AD92-E888F69598AC}"/>
   </bookViews>
   <sheets>
     <sheet name="load" sheetId="5" r:id="rId1"/>
@@ -12734,120 +12734,408 @@
       <c r="A3" s="1">
         <v>0</v>
       </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>4.1666666666666664E-2</v>
       </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>8.3333333333333301E-2</v>
       </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>0.125</v>
       </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>0.16666666666666699</v>
       </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>0.20833333333333301</v>
       </c>
+      <c r="V8">
+        <v>9.4083203000000001E-3</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <v>1.6259327100000002E-2</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>0.25</v>
       </c>
+      <c r="V9">
+        <v>4.39345742E-2</v>
+      </c>
+      <c r="W9">
+        <v>0</v>
+      </c>
+      <c r="X9">
+        <v>4.9704414100000004E-2</v>
+      </c>
+      <c r="Y9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>0.29166666666666702</v>
       </c>
+      <c r="V10">
+        <v>9.1964718799999998E-2</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>9.6043515600000004E-2</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>0.33333333333333298</v>
       </c>
+      <c r="V11">
+        <v>0.1349729844</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+      <c r="X11">
+        <v>0.141470125</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>0.375</v>
       </c>
+      <c r="V12">
+        <v>0.16872196880000001</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>0.18009662500000001</v>
+      </c>
+      <c r="Y12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>0.41666666666666702</v>
       </c>
+      <c r="V13">
+        <v>0.19263135939999998</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <v>0.20747953129999999</v>
+      </c>
+      <c r="Y13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>0.45833333333333298</v>
       </c>
+      <c r="V14">
+        <v>0.20567318749999999</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0.22436475</v>
+      </c>
+      <c r="Y14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>0.5</v>
       </c>
+      <c r="V15">
+        <v>0.20856379689999999</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>0.23317234380000001</v>
+      </c>
+      <c r="Y15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:39" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>0.54166666666666696</v>
       </c>
+      <c r="V16">
+        <v>0.20429056249999999</v>
+      </c>
+      <c r="W16">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>0.23407293749999999</v>
+      </c>
+      <c r="Y16">
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>0.58333333333333304</v>
       </c>
+      <c r="V17">
+        <v>0.19125948439999998</v>
+      </c>
+      <c r="W17">
+        <v>0</v>
+      </c>
+      <c r="X17">
+        <v>0.22401164060000001</v>
+      </c>
+      <c r="Y17">
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>0.625</v>
       </c>
+      <c r="V18">
+        <v>0.16881509380000001</v>
+      </c>
+      <c r="W18">
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <v>0.20421040630000001</v>
+      </c>
+      <c r="Y18">
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A19" s="1">
         <v>0.66666666666666696</v>
       </c>
+      <c r="V19">
+        <v>0.13611562499999999</v>
+      </c>
+      <c r="W19">
+        <v>0</v>
+      </c>
+      <c r="X19">
+        <v>0.17339570310000002</v>
+      </c>
+      <c r="Y19">
+        <v>0</v>
+      </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A20" s="1">
         <v>0.70833333333333304</v>
       </c>
+      <c r="V20">
+        <v>9.41819297E-2</v>
+      </c>
+      <c r="W20">
+        <v>0</v>
+      </c>
+      <c r="X20">
+        <v>0.13052409379999999</v>
+      </c>
+      <c r="Y20">
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A21" s="1">
         <v>0.75</v>
       </c>
+      <c r="V21">
+        <v>4.85839219E-2</v>
+      </c>
+      <c r="W21">
+        <v>0</v>
+      </c>
+      <c r="X21">
+        <v>8.4502382800000012E-2</v>
+      </c>
+      <c r="Y21">
+        <v>0</v>
+      </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A22" s="1">
         <v>0.79166666666666696</v>
       </c>
+      <c r="V22">
+        <v>2.0931398399999999E-2</v>
+      </c>
+      <c r="W22">
+        <v>0</v>
+      </c>
+      <c r="X22">
+        <v>4.8002406300000001E-2</v>
+      </c>
+      <c r="Y22">
+        <v>0</v>
+      </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A23" s="1">
         <v>0.83333333333333304</v>
       </c>
+      <c r="V23">
+        <v>0</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>0</v>
+      </c>
+      <c r="Y23">
+        <v>0</v>
+      </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A24" s="1">
         <v>0.875</v>
       </c>
+      <c r="V24">
+        <v>0</v>
+      </c>
+      <c r="W24">
+        <v>0</v>
+      </c>
+      <c r="X24">
+        <v>0</v>
+      </c>
+      <c r="Y24">
+        <v>0</v>
+      </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A25" s="1">
         <v>0.91666666666666696</v>
       </c>
+      <c r="V25">
+        <v>0</v>
+      </c>
+      <c r="W25">
+        <v>0</v>
+      </c>
+      <c r="X25">
+        <v>0</v>
+      </c>
+      <c r="Y25">
+        <v>0</v>
+      </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A26" s="1">
         <v>0.95833333333333304</v>
+      </c>
+      <c r="V26">
+        <v>0</v>
+      </c>
+      <c r="W26">
+        <v>0</v>
+      </c>
+      <c r="X26">
+        <v>0</v>
+      </c>
+      <c r="Y26">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>